<commit_message>
Remove generated reports and update gitignore
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SanjaY\eclipse\eclipse\Workspace\ApiFramework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C4DBC4-4980-468E-BB98-730262A40C2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF82E2A-571F-4EA5-8828-2B0046D956E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4008" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,9 +81,6 @@
     <t>Sanjay</t>
   </si>
   <si>
-    <t>Maxpayne@3</t>
-  </si>
-  <si>
     <t>Mr</t>
   </si>
   <si>
@@ -105,7 +102,10 @@
     <t>Karnataka</t>
   </si>
   <si>
-    <t>skgkkah@hkh.com</t>
+    <t>sanjay@gmail.com</t>
+  </si>
+  <si>
+    <t>Password@3</t>
   </si>
 </sst>
 </file>
@@ -527,37 +527,37 @@
         <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="L2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M2" s="2">
         <v>560001</v>
@@ -578,6 +578,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{65EF50F0-C8B6-47E8-B898-8A52055C3115}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{53026CB3-6D5D-4CE8-B27D-55A8A298113A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>